<commit_message>
logical structure code 20260203 v1
</commit_message>
<xml_diff>
--- a/logical_structure_analysis/statistic_files/embed_summary.xlsx
+++ b/logical_structure_analysis/statistic_files/embed_summary.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J151"/>
+  <dimension ref="A1:J91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -514,10 +514,10 @@
         <v>300</v>
       </c>
       <c r="H2" t="n">
-        <v>250</v>
+        <v>223</v>
       </c>
       <c r="I2" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.7433333333333333</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -593,13 +593,13 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0.8333333333333334</v>
+        <v>0</v>
       </c>
       <c r="J4" t="inlineStr"/>
     </row>
@@ -633,13 +633,13 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>223</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>0.7433333333333333</v>
       </c>
       <c r="J5" t="inlineStr"/>
     </row>
@@ -716,10 +716,10 @@
         <v>300</v>
       </c>
       <c r="H7" t="n">
-        <v>250</v>
+        <v>221</v>
       </c>
       <c r="I7" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.7366666666666667</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -795,13 +795,13 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>0.8333333333333334</v>
+        <v>0</v>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
@@ -835,13 +835,13 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>221</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>0.7366666666666667</v>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
@@ -918,10 +918,10 @@
         <v>300</v>
       </c>
       <c r="H12" t="n">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="I12" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.8566666666666667</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -997,13 +997,13 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>0.8333333333333334</v>
+        <v>0</v>
       </c>
       <c r="J14" t="inlineStr"/>
     </row>
@@ -1037,13 +1037,13 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>257</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>0.8566666666666667</v>
       </c>
       <c r="J15" t="inlineStr"/>
     </row>
@@ -1120,10 +1120,10 @@
         <v>300</v>
       </c>
       <c r="H17" t="n">
-        <v>250</v>
+        <v>221</v>
       </c>
       <c r="I17" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.7366666666666667</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1199,13 +1199,13 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>0.8333333333333334</v>
+        <v>0</v>
       </c>
       <c r="J19" t="inlineStr"/>
     </row>
@@ -1239,13 +1239,13 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>221</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>0.7366666666666667</v>
       </c>
       <c r="J20" t="inlineStr"/>
     </row>
@@ -1322,10 +1322,10 @@
         <v>300</v>
       </c>
       <c r="H22" t="n">
-        <v>250</v>
+        <v>221</v>
       </c>
       <c r="I22" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.7366666666666667</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1401,13 +1401,13 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>0.8333333333333334</v>
+        <v>0</v>
       </c>
       <c r="J24" t="inlineStr"/>
     </row>
@@ -1441,13 +1441,13 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>221</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>0.7366666666666667</v>
       </c>
       <c r="J25" t="inlineStr"/>
     </row>
@@ -1603,13 +1603,13 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>237</v>
+        <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>0.79</v>
+        <v>0</v>
       </c>
       <c r="J29" t="inlineStr"/>
     </row>
@@ -1643,13 +1643,13 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>237</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
+        <v>0.79</v>
       </c>
       <c r="J30" t="inlineStr"/>
     </row>
@@ -1726,10 +1726,10 @@
         <v>300</v>
       </c>
       <c r="H32" t="n">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="I32" t="n">
-        <v>0.8466666666666667</v>
+        <v>0.86</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1805,13 +1805,13 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>254</v>
+        <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>0.8466666666666667</v>
+        <v>0</v>
       </c>
       <c r="J34" t="inlineStr"/>
     </row>
@@ -1845,13 +1845,13 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>258</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>0.86</v>
       </c>
       <c r="J35" t="inlineStr"/>
     </row>
@@ -1928,10 +1928,10 @@
         <v>300</v>
       </c>
       <c r="H37" t="n">
-        <v>253</v>
+        <v>262</v>
       </c>
       <c r="I37" t="n">
-        <v>0.8433333333333334</v>
+        <v>0.8733333333333333</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -2007,13 +2007,13 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>253</v>
+        <v>0</v>
       </c>
       <c r="I39" t="n">
-        <v>0.8433333333333334</v>
+        <v>0</v>
       </c>
       <c r="J39" t="inlineStr"/>
     </row>
@@ -2047,13 +2047,13 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>262</v>
       </c>
       <c r="I40" t="n">
-        <v>0</v>
+        <v>0.8733333333333333</v>
       </c>
       <c r="J40" t="inlineStr"/>
     </row>
@@ -2130,10 +2130,10 @@
         <v>300</v>
       </c>
       <c r="H42" t="n">
-        <v>246</v>
+        <v>259</v>
       </c>
       <c r="I42" t="n">
-        <v>0.82</v>
+        <v>0.8633333333333333</v>
       </c>
       <c r="J42" t="n">
         <v>0</v>
@@ -2209,13 +2209,13 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H44" t="n">
-        <v>246</v>
+        <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>0.82</v>
+        <v>0</v>
       </c>
       <c r="J44" t="inlineStr"/>
     </row>
@@ -2249,13 +2249,13 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H45" t="n">
-        <v>0</v>
+        <v>259</v>
       </c>
       <c r="I45" t="n">
-        <v>0</v>
+        <v>0.8633333333333333</v>
       </c>
       <c r="J45" t="inlineStr"/>
     </row>
@@ -2332,10 +2332,10 @@
         <v>300</v>
       </c>
       <c r="H47" t="n">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="I47" t="n">
-        <v>0.84</v>
+        <v>0.87</v>
       </c>
       <c r="J47" t="n">
         <v>0</v>
@@ -2411,13 +2411,13 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H49" t="n">
-        <v>252</v>
+        <v>0</v>
       </c>
       <c r="I49" t="n">
-        <v>0.84</v>
+        <v>0</v>
       </c>
       <c r="J49" t="inlineStr"/>
     </row>
@@ -2451,13 +2451,13 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H50" t="n">
-        <v>0</v>
+        <v>261</v>
       </c>
       <c r="I50" t="n">
-        <v>0</v>
+        <v>0.87</v>
       </c>
       <c r="J50" t="inlineStr"/>
     </row>
@@ -2534,10 +2534,10 @@
         <v>300</v>
       </c>
       <c r="H52" t="n">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="I52" t="n">
-        <v>0.8066666666666666</v>
+        <v>0.7566666666666667</v>
       </c>
       <c r="J52" t="n">
         <v>0</v>
@@ -2613,13 +2613,13 @@
         </is>
       </c>
       <c r="G54" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H54" t="n">
-        <v>242</v>
+        <v>0</v>
       </c>
       <c r="I54" t="n">
-        <v>0.8066666666666666</v>
+        <v>0</v>
       </c>
       <c r="J54" t="inlineStr"/>
     </row>
@@ -2653,13 +2653,13 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H55" t="n">
-        <v>0</v>
+        <v>227</v>
       </c>
       <c r="I55" t="n">
-        <v>0</v>
+        <v>0.7566666666666667</v>
       </c>
       <c r="J55" t="inlineStr"/>
     </row>
@@ -2736,10 +2736,10 @@
         <v>300</v>
       </c>
       <c r="H57" t="n">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="I57" t="n">
-        <v>0.8666666666666667</v>
+        <v>0.88</v>
       </c>
       <c r="J57" t="n">
         <v>0</v>
@@ -2815,13 +2815,13 @@
         </is>
       </c>
       <c r="G59" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H59" t="n">
-        <v>260</v>
+        <v>0</v>
       </c>
       <c r="I59" t="n">
-        <v>0.8666666666666667</v>
+        <v>0</v>
       </c>
       <c r="J59" t="inlineStr"/>
     </row>
@@ -2855,13 +2855,13 @@
         </is>
       </c>
       <c r="G60" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H60" t="n">
-        <v>0</v>
+        <v>264</v>
       </c>
       <c r="I60" t="n">
-        <v>0</v>
+        <v>0.88</v>
       </c>
       <c r="J60" t="inlineStr"/>
     </row>
@@ -3017,13 +3017,13 @@
         </is>
       </c>
       <c r="G64" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H64" t="n">
-        <v>252</v>
+        <v>0</v>
       </c>
       <c r="I64" t="n">
-        <v>0.84</v>
+        <v>0</v>
       </c>
       <c r="J64" t="inlineStr"/>
     </row>
@@ -3057,13 +3057,13 @@
         </is>
       </c>
       <c r="G65" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H65" t="n">
-        <v>0</v>
+        <v>252</v>
       </c>
       <c r="I65" t="n">
-        <v>0</v>
+        <v>0.84</v>
       </c>
       <c r="J65" t="inlineStr"/>
     </row>
@@ -3219,13 +3219,13 @@
         </is>
       </c>
       <c r="G69" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H69" t="n">
-        <v>257</v>
+        <v>0</v>
       </c>
       <c r="I69" t="n">
-        <v>0.8566666666666667</v>
+        <v>0</v>
       </c>
       <c r="J69" t="inlineStr"/>
     </row>
@@ -3259,13 +3259,13 @@
         </is>
       </c>
       <c r="G70" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H70" t="n">
-        <v>0</v>
+        <v>257</v>
       </c>
       <c r="I70" t="n">
-        <v>0</v>
+        <v>0.8566666666666667</v>
       </c>
       <c r="J70" t="inlineStr"/>
     </row>
@@ -3342,10 +3342,10 @@
         <v>300</v>
       </c>
       <c r="H72" t="n">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="I72" t="n">
-        <v>0.85</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="J72" t="n">
         <v>0</v>
@@ -3421,13 +3421,13 @@
         </is>
       </c>
       <c r="G74" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H74" t="n">
-        <v>255</v>
+        <v>0</v>
       </c>
       <c r="I74" t="n">
-        <v>0.85</v>
+        <v>0</v>
       </c>
       <c r="J74" t="inlineStr"/>
     </row>
@@ -3461,13 +3461,13 @@
         </is>
       </c>
       <c r="G75" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H75" t="n">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="I75" t="n">
-        <v>0</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="J75" t="inlineStr"/>
     </row>
@@ -3544,10 +3544,10 @@
         <v>300</v>
       </c>
       <c r="H77" t="n">
-        <v>232</v>
+        <v>219</v>
       </c>
       <c r="I77" t="n">
-        <v>0.7733333333333333</v>
+        <v>0.73</v>
       </c>
       <c r="J77" t="n">
         <v>0</v>
@@ -3623,13 +3623,13 @@
         </is>
       </c>
       <c r="G79" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H79" t="n">
-        <v>232</v>
+        <v>0</v>
       </c>
       <c r="I79" t="n">
-        <v>0.7733333333333333</v>
+        <v>0</v>
       </c>
       <c r="J79" t="inlineStr"/>
     </row>
@@ -3663,13 +3663,13 @@
         </is>
       </c>
       <c r="G80" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H80" t="n">
-        <v>0</v>
+        <v>219</v>
       </c>
       <c r="I80" t="n">
-        <v>0</v>
+        <v>0.73</v>
       </c>
       <c r="J80" t="inlineStr"/>
     </row>
@@ -3746,10 +3746,10 @@
         <v>300</v>
       </c>
       <c r="H82" t="n">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="I82" t="n">
-        <v>0.8366666666666667</v>
+        <v>0.8566666666666667</v>
       </c>
       <c r="J82" t="n">
         <v>0</v>
@@ -3825,13 +3825,13 @@
         </is>
       </c>
       <c r="G84" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H84" t="n">
-        <v>251</v>
+        <v>0</v>
       </c>
       <c r="I84" t="n">
-        <v>0.8366666666666667</v>
+        <v>0</v>
       </c>
       <c r="J84" t="inlineStr"/>
     </row>
@@ -3865,13 +3865,13 @@
         </is>
       </c>
       <c r="G85" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H85" t="n">
-        <v>0</v>
+        <v>257</v>
       </c>
       <c r="I85" t="n">
-        <v>0</v>
+        <v>0.8566666666666667</v>
       </c>
       <c r="J85" t="inlineStr"/>
     </row>
@@ -3918,7 +3918,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ProntoQA</t>
+          <t>ProofWriter</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -3936,7 +3936,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>embed_results/LogicalDeduction/k4/ProntoQA__LogicalDeduction_dev_k4_icl.json</t>
+          <t>embed_results/LogicalDeduction/k4/ProofWriter__LogicalDeduction_dev_k4_icl.json</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -3948,10 +3948,10 @@
         <v>300</v>
       </c>
       <c r="H87" t="n">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="I87" t="n">
-        <v>0.8533333333333334</v>
+        <v>0.8566666666666667</v>
       </c>
       <c r="J87" t="n">
         <v>0</v>
@@ -3960,7 +3960,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ProntoQA</t>
+          <t>ProofWriter</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>embed_results/LogicalDeduction/k4/ProntoQA__LogicalDeduction_dev_k4_icl.json</t>
+          <t>embed_results/LogicalDeduction/k4/ProofWriter__LogicalDeduction_dev_k4_icl.json</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -4000,7 +4000,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ProntoQA</t>
+          <t>ProofWriter</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4018,7 +4018,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>embed_results/LogicalDeduction/k4/ProntoQA__LogicalDeduction_dev_k4_icl.json</t>
+          <t>embed_results/LogicalDeduction/k4/ProofWriter__LogicalDeduction_dev_k4_icl.json</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -4027,20 +4027,20 @@
         </is>
       </c>
       <c r="G89" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H89" t="n">
-        <v>256</v>
+        <v>0</v>
       </c>
       <c r="I89" t="n">
-        <v>0.8533333333333334</v>
+        <v>0</v>
       </c>
       <c r="J89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ProntoQA</t>
+          <t>ProofWriter</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4058,7 +4058,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>embed_results/LogicalDeduction/k4/ProntoQA__LogicalDeduction_dev_k4_icl.json</t>
+          <t>embed_results/LogicalDeduction/k4/ProofWriter__LogicalDeduction_dev_k4_icl.json</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -4067,20 +4067,20 @@
         </is>
       </c>
       <c r="G90" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H90" t="n">
-        <v>0</v>
+        <v>257</v>
       </c>
       <c r="I90" t="n">
-        <v>0</v>
+        <v>0.8566666666666667</v>
       </c>
       <c r="J90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ProntoQA</t>
+          <t>ProofWriter</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4098,7 +4098,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>embed_results/LogicalDeduction/k4/ProntoQA__LogicalDeduction_dev_k4_icl.json</t>
+          <t>embed_results/LogicalDeduction/k4/ProofWriter__LogicalDeduction_dev_k4_icl.json</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -4116,2430 +4116,6 @@
         <v>0</v>
       </c>
       <c r="J91" t="inlineStr"/>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>ProofWriter</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D92" t="n">
-        <v>4</v>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k4/ProofWriter__LogicalDeduction_dev_k4_icl.json</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="G92" t="n">
-        <v>300</v>
-      </c>
-      <c r="H92" t="n">
-        <v>254</v>
-      </c>
-      <c r="I92" t="n">
-        <v>0.8466666666666667</v>
-      </c>
-      <c r="J92" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>ProofWriter</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D93" t="n">
-        <v>4</v>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k4/ProofWriter__LogicalDeduction_dev_k4_icl.json</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>Block</t>
-        </is>
-      </c>
-      <c r="G93" t="n">
-        <v>0</v>
-      </c>
-      <c r="H93" t="n">
-        <v>0</v>
-      </c>
-      <c r="I93" t="n">
-        <v>0</v>
-      </c>
-      <c r="J93" t="inlineStr"/>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>ProofWriter</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D94" t="n">
-        <v>4</v>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k4/ProofWriter__LogicalDeduction_dev_k4_icl.json</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>Chain</t>
-        </is>
-      </c>
-      <c r="G94" t="n">
-        <v>300</v>
-      </c>
-      <c r="H94" t="n">
-        <v>254</v>
-      </c>
-      <c r="I94" t="n">
-        <v>0.8466666666666667</v>
-      </c>
-      <c r="J94" t="inlineStr"/>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>ProofWriter</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D95" t="n">
-        <v>4</v>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k4/ProofWriter__LogicalDeduction_dev_k4_icl.json</t>
-        </is>
-      </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="G95" t="n">
-        <v>0</v>
-      </c>
-      <c r="H95" t="n">
-        <v>0</v>
-      </c>
-      <c r="I95" t="n">
-        <v>0</v>
-      </c>
-      <c r="J95" t="inlineStr"/>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>ProofWriter</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D96" t="n">
-        <v>4</v>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k4/ProofWriter__LogicalDeduction_dev_k4_icl.json</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>Y-shaped</t>
-        </is>
-      </c>
-      <c r="G96" t="n">
-        <v>0</v>
-      </c>
-      <c r="H96" t="n">
-        <v>0</v>
-      </c>
-      <c r="I96" t="n">
-        <v>0</v>
-      </c>
-      <c r="J96" t="inlineStr"/>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>gsm8k</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D97" t="n">
-        <v>4</v>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k4/gsm8k__LogicalDeduction_dev_k4_icl.json</t>
-        </is>
-      </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="G97" t="n">
-        <v>300</v>
-      </c>
-      <c r="H97" t="n">
-        <v>252</v>
-      </c>
-      <c r="I97" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="J97" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>gsm8k</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D98" t="n">
-        <v>4</v>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k4/gsm8k__LogicalDeduction_dev_k4_icl.json</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>Block</t>
-        </is>
-      </c>
-      <c r="G98" t="n">
-        <v>0</v>
-      </c>
-      <c r="H98" t="n">
-        <v>0</v>
-      </c>
-      <c r="I98" t="n">
-        <v>0</v>
-      </c>
-      <c r="J98" t="inlineStr"/>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>gsm8k</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D99" t="n">
-        <v>4</v>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k4/gsm8k__LogicalDeduction_dev_k4_icl.json</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>Chain</t>
-        </is>
-      </c>
-      <c r="G99" t="n">
-        <v>300</v>
-      </c>
-      <c r="H99" t="n">
-        <v>252</v>
-      </c>
-      <c r="I99" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="J99" t="inlineStr"/>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>gsm8k</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D100" t="n">
-        <v>4</v>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k4/gsm8k__LogicalDeduction_dev_k4_icl.json</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="G100" t="n">
-        <v>0</v>
-      </c>
-      <c r="H100" t="n">
-        <v>0</v>
-      </c>
-      <c r="I100" t="n">
-        <v>0</v>
-      </c>
-      <c r="J100" t="inlineStr"/>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>gsm8k</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D101" t="n">
-        <v>4</v>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k4/gsm8k__LogicalDeduction_dev_k4_icl.json</t>
-        </is>
-      </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>Y-shaped</t>
-        </is>
-      </c>
-      <c r="G101" t="n">
-        <v>0</v>
-      </c>
-      <c r="H101" t="n">
-        <v>0</v>
-      </c>
-      <c r="I101" t="n">
-        <v>0</v>
-      </c>
-      <c r="J101" t="inlineStr"/>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>AR-LSAT</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D102" t="n">
-        <v>6</v>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/AR-LSAT__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="G102" t="n">
-        <v>300</v>
-      </c>
-      <c r="H102" t="n">
-        <v>232</v>
-      </c>
-      <c r="I102" t="n">
-        <v>0.7733333333333333</v>
-      </c>
-      <c r="J102" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>AR-LSAT</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D103" t="n">
-        <v>6</v>
-      </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/AR-LSAT__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>Block</t>
-        </is>
-      </c>
-      <c r="G103" t="n">
-        <v>0</v>
-      </c>
-      <c r="H103" t="n">
-        <v>0</v>
-      </c>
-      <c r="I103" t="n">
-        <v>0</v>
-      </c>
-      <c r="J103" t="inlineStr"/>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>AR-LSAT</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D104" t="n">
-        <v>6</v>
-      </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/AR-LSAT__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>Chain</t>
-        </is>
-      </c>
-      <c r="G104" t="n">
-        <v>300</v>
-      </c>
-      <c r="H104" t="n">
-        <v>232</v>
-      </c>
-      <c r="I104" t="n">
-        <v>0.7733333333333333</v>
-      </c>
-      <c r="J104" t="inlineStr"/>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>AR-LSAT</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D105" t="n">
-        <v>6</v>
-      </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/AR-LSAT__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="G105" t="n">
-        <v>0</v>
-      </c>
-      <c r="H105" t="n">
-        <v>0</v>
-      </c>
-      <c r="I105" t="n">
-        <v>0</v>
-      </c>
-      <c r="J105" t="inlineStr"/>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>AR-LSAT</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D106" t="n">
-        <v>6</v>
-      </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/AR-LSAT__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>Y-shaped</t>
-        </is>
-      </c>
-      <c r="G106" t="n">
-        <v>0</v>
-      </c>
-      <c r="H106" t="n">
-        <v>0</v>
-      </c>
-      <c r="I106" t="n">
-        <v>0</v>
-      </c>
-      <c r="J106" t="inlineStr"/>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>FOLIO</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D107" t="n">
-        <v>6</v>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/FOLIO__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="G107" t="n">
-        <v>300</v>
-      </c>
-      <c r="H107" t="n">
-        <v>255</v>
-      </c>
-      <c r="I107" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="J107" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>FOLIO</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D108" t="n">
-        <v>6</v>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/FOLIO__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>Block</t>
-        </is>
-      </c>
-      <c r="G108" t="n">
-        <v>0</v>
-      </c>
-      <c r="H108" t="n">
-        <v>0</v>
-      </c>
-      <c r="I108" t="n">
-        <v>0</v>
-      </c>
-      <c r="J108" t="inlineStr"/>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>FOLIO</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D109" t="n">
-        <v>6</v>
-      </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/FOLIO__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>Chain</t>
-        </is>
-      </c>
-      <c r="G109" t="n">
-        <v>300</v>
-      </c>
-      <c r="H109" t="n">
-        <v>255</v>
-      </c>
-      <c r="I109" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="J109" t="inlineStr"/>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>FOLIO</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D110" t="n">
-        <v>6</v>
-      </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/FOLIO__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="G110" t="n">
-        <v>0</v>
-      </c>
-      <c r="H110" t="n">
-        <v>0</v>
-      </c>
-      <c r="I110" t="n">
-        <v>0</v>
-      </c>
-      <c r="J110" t="inlineStr"/>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>FOLIO</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D111" t="n">
-        <v>6</v>
-      </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/FOLIO__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>Y-shaped</t>
-        </is>
-      </c>
-      <c r="G111" t="n">
-        <v>0</v>
-      </c>
-      <c r="H111" t="n">
-        <v>0</v>
-      </c>
-      <c r="I111" t="n">
-        <v>0</v>
-      </c>
-      <c r="J111" t="inlineStr"/>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>ProntoQA</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D112" t="n">
-        <v>6</v>
-      </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/ProntoQA__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F112" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="G112" t="n">
-        <v>300</v>
-      </c>
-      <c r="H112" t="n">
-        <v>254</v>
-      </c>
-      <c r="I112" t="n">
-        <v>0.8466666666666667</v>
-      </c>
-      <c r="J112" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>ProntoQA</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D113" t="n">
-        <v>6</v>
-      </c>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/ProntoQA__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F113" t="inlineStr">
-        <is>
-          <t>Block</t>
-        </is>
-      </c>
-      <c r="G113" t="n">
-        <v>0</v>
-      </c>
-      <c r="H113" t="n">
-        <v>0</v>
-      </c>
-      <c r="I113" t="n">
-        <v>0</v>
-      </c>
-      <c r="J113" t="inlineStr"/>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>ProntoQA</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D114" t="n">
-        <v>6</v>
-      </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/ProntoQA__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t>Chain</t>
-        </is>
-      </c>
-      <c r="G114" t="n">
-        <v>300</v>
-      </c>
-      <c r="H114" t="n">
-        <v>254</v>
-      </c>
-      <c r="I114" t="n">
-        <v>0.8466666666666667</v>
-      </c>
-      <c r="J114" t="inlineStr"/>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>ProntoQA</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D115" t="n">
-        <v>6</v>
-      </c>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/ProntoQA__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="G115" t="n">
-        <v>0</v>
-      </c>
-      <c r="H115" t="n">
-        <v>0</v>
-      </c>
-      <c r="I115" t="n">
-        <v>0</v>
-      </c>
-      <c r="J115" t="inlineStr"/>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>ProntoQA</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D116" t="n">
-        <v>6</v>
-      </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/ProntoQA__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>Y-shaped</t>
-        </is>
-      </c>
-      <c r="G116" t="n">
-        <v>0</v>
-      </c>
-      <c r="H116" t="n">
-        <v>0</v>
-      </c>
-      <c r="I116" t="n">
-        <v>0</v>
-      </c>
-      <c r="J116" t="inlineStr"/>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>ProofWriter</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D117" t="n">
-        <v>6</v>
-      </c>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/ProofWriter__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F117" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="G117" t="n">
-        <v>300</v>
-      </c>
-      <c r="H117" t="n">
-        <v>254</v>
-      </c>
-      <c r="I117" t="n">
-        <v>0.8466666666666667</v>
-      </c>
-      <c r="J117" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>ProofWriter</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D118" t="n">
-        <v>6</v>
-      </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/ProofWriter__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F118" t="inlineStr">
-        <is>
-          <t>Block</t>
-        </is>
-      </c>
-      <c r="G118" t="n">
-        <v>0</v>
-      </c>
-      <c r="H118" t="n">
-        <v>0</v>
-      </c>
-      <c r="I118" t="n">
-        <v>0</v>
-      </c>
-      <c r="J118" t="inlineStr"/>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>ProofWriter</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D119" t="n">
-        <v>6</v>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/ProofWriter__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>Chain</t>
-        </is>
-      </c>
-      <c r="G119" t="n">
-        <v>300</v>
-      </c>
-      <c r="H119" t="n">
-        <v>254</v>
-      </c>
-      <c r="I119" t="n">
-        <v>0.8466666666666667</v>
-      </c>
-      <c r="J119" t="inlineStr"/>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>ProofWriter</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D120" t="n">
-        <v>6</v>
-      </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/ProofWriter__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="G120" t="n">
-        <v>0</v>
-      </c>
-      <c r="H120" t="n">
-        <v>0</v>
-      </c>
-      <c r="I120" t="n">
-        <v>0</v>
-      </c>
-      <c r="J120" t="inlineStr"/>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>ProofWriter</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D121" t="n">
-        <v>6</v>
-      </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/ProofWriter__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>Y-shaped</t>
-        </is>
-      </c>
-      <c r="G121" t="n">
-        <v>0</v>
-      </c>
-      <c r="H121" t="n">
-        <v>0</v>
-      </c>
-      <c r="I121" t="n">
-        <v>0</v>
-      </c>
-      <c r="J121" t="inlineStr"/>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>gsm8k</t>
-        </is>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D122" t="n">
-        <v>6</v>
-      </c>
-      <c r="E122" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/gsm8k__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="G122" t="n">
-        <v>300</v>
-      </c>
-      <c r="H122" t="n">
-        <v>254</v>
-      </c>
-      <c r="I122" t="n">
-        <v>0.8466666666666667</v>
-      </c>
-      <c r="J122" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>gsm8k</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D123" t="n">
-        <v>6</v>
-      </c>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/gsm8k__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F123" t="inlineStr">
-        <is>
-          <t>Block</t>
-        </is>
-      </c>
-      <c r="G123" t="n">
-        <v>0</v>
-      </c>
-      <c r="H123" t="n">
-        <v>0</v>
-      </c>
-      <c r="I123" t="n">
-        <v>0</v>
-      </c>
-      <c r="J123" t="inlineStr"/>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>gsm8k</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D124" t="n">
-        <v>6</v>
-      </c>
-      <c r="E124" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/gsm8k__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F124" t="inlineStr">
-        <is>
-          <t>Chain</t>
-        </is>
-      </c>
-      <c r="G124" t="n">
-        <v>300</v>
-      </c>
-      <c r="H124" t="n">
-        <v>254</v>
-      </c>
-      <c r="I124" t="n">
-        <v>0.8466666666666667</v>
-      </c>
-      <c r="J124" t="inlineStr"/>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>gsm8k</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D125" t="n">
-        <v>6</v>
-      </c>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/gsm8k__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="G125" t="n">
-        <v>0</v>
-      </c>
-      <c r="H125" t="n">
-        <v>0</v>
-      </c>
-      <c r="I125" t="n">
-        <v>0</v>
-      </c>
-      <c r="J125" t="inlineStr"/>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>gsm8k</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D126" t="n">
-        <v>6</v>
-      </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/gsm8k__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>Y-shaped</t>
-        </is>
-      </c>
-      <c r="G126" t="n">
-        <v>0</v>
-      </c>
-      <c r="H126" t="n">
-        <v>0</v>
-      </c>
-      <c r="I126" t="n">
-        <v>0</v>
-      </c>
-      <c r="J126" t="inlineStr"/>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>AR-LSAT</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D127" t="n">
-        <v>8</v>
-      </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/AR-LSAT__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="G127" t="n">
-        <v>300</v>
-      </c>
-      <c r="H127" t="n">
-        <v>242</v>
-      </c>
-      <c r="I127" t="n">
-        <v>0.8066666666666666</v>
-      </c>
-      <c r="J127" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>AR-LSAT</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D128" t="n">
-        <v>8</v>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/AR-LSAT__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F128" t="inlineStr">
-        <is>
-          <t>Block</t>
-        </is>
-      </c>
-      <c r="G128" t="n">
-        <v>0</v>
-      </c>
-      <c r="H128" t="n">
-        <v>0</v>
-      </c>
-      <c r="I128" t="n">
-        <v>0</v>
-      </c>
-      <c r="J128" t="inlineStr"/>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>AR-LSAT</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D129" t="n">
-        <v>8</v>
-      </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/AR-LSAT__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F129" t="inlineStr">
-        <is>
-          <t>Chain</t>
-        </is>
-      </c>
-      <c r="G129" t="n">
-        <v>300</v>
-      </c>
-      <c r="H129" t="n">
-        <v>242</v>
-      </c>
-      <c r="I129" t="n">
-        <v>0.8066666666666666</v>
-      </c>
-      <c r="J129" t="inlineStr"/>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>AR-LSAT</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D130" t="n">
-        <v>8</v>
-      </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/AR-LSAT__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F130" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="G130" t="n">
-        <v>0</v>
-      </c>
-      <c r="H130" t="n">
-        <v>0</v>
-      </c>
-      <c r="I130" t="n">
-        <v>0</v>
-      </c>
-      <c r="J130" t="inlineStr"/>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>AR-LSAT</t>
-        </is>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D131" t="n">
-        <v>8</v>
-      </c>
-      <c r="E131" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/AR-LSAT__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F131" t="inlineStr">
-        <is>
-          <t>Y-shaped</t>
-        </is>
-      </c>
-      <c r="G131" t="n">
-        <v>0</v>
-      </c>
-      <c r="H131" t="n">
-        <v>0</v>
-      </c>
-      <c r="I131" t="n">
-        <v>0</v>
-      </c>
-      <c r="J131" t="inlineStr"/>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>FOLIO</t>
-        </is>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D132" t="n">
-        <v>8</v>
-      </c>
-      <c r="E132" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/FOLIO__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F132" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="G132" t="n">
-        <v>300</v>
-      </c>
-      <c r="H132" t="n">
-        <v>244</v>
-      </c>
-      <c r="I132" t="n">
-        <v>0.8133333333333334</v>
-      </c>
-      <c r="J132" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>FOLIO</t>
-        </is>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D133" t="n">
-        <v>8</v>
-      </c>
-      <c r="E133" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/FOLIO__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F133" t="inlineStr">
-        <is>
-          <t>Block</t>
-        </is>
-      </c>
-      <c r="G133" t="n">
-        <v>0</v>
-      </c>
-      <c r="H133" t="n">
-        <v>0</v>
-      </c>
-      <c r="I133" t="n">
-        <v>0</v>
-      </c>
-      <c r="J133" t="inlineStr"/>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>FOLIO</t>
-        </is>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D134" t="n">
-        <v>8</v>
-      </c>
-      <c r="E134" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/FOLIO__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F134" t="inlineStr">
-        <is>
-          <t>Chain</t>
-        </is>
-      </c>
-      <c r="G134" t="n">
-        <v>300</v>
-      </c>
-      <c r="H134" t="n">
-        <v>244</v>
-      </c>
-      <c r="I134" t="n">
-        <v>0.8133333333333334</v>
-      </c>
-      <c r="J134" t="inlineStr"/>
-    </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>FOLIO</t>
-        </is>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D135" t="n">
-        <v>8</v>
-      </c>
-      <c r="E135" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/FOLIO__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F135" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="G135" t="n">
-        <v>0</v>
-      </c>
-      <c r="H135" t="n">
-        <v>0</v>
-      </c>
-      <c r="I135" t="n">
-        <v>0</v>
-      </c>
-      <c r="J135" t="inlineStr"/>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>FOLIO</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D136" t="n">
-        <v>8</v>
-      </c>
-      <c r="E136" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/FOLIO__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F136" t="inlineStr">
-        <is>
-          <t>Y-shaped</t>
-        </is>
-      </c>
-      <c r="G136" t="n">
-        <v>0</v>
-      </c>
-      <c r="H136" t="n">
-        <v>0</v>
-      </c>
-      <c r="I136" t="n">
-        <v>0</v>
-      </c>
-      <c r="J136" t="inlineStr"/>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>ProntoQA</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D137" t="n">
-        <v>8</v>
-      </c>
-      <c r="E137" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/ProntoQA__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F137" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="G137" t="n">
-        <v>300</v>
-      </c>
-      <c r="H137" t="n">
-        <v>251</v>
-      </c>
-      <c r="I137" t="n">
-        <v>0.8366666666666667</v>
-      </c>
-      <c r="J137" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>ProntoQA</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D138" t="n">
-        <v>8</v>
-      </c>
-      <c r="E138" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/ProntoQA__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F138" t="inlineStr">
-        <is>
-          <t>Block</t>
-        </is>
-      </c>
-      <c r="G138" t="n">
-        <v>0</v>
-      </c>
-      <c r="H138" t="n">
-        <v>0</v>
-      </c>
-      <c r="I138" t="n">
-        <v>0</v>
-      </c>
-      <c r="J138" t="inlineStr"/>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>ProntoQA</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D139" t="n">
-        <v>8</v>
-      </c>
-      <c r="E139" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/ProntoQA__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F139" t="inlineStr">
-        <is>
-          <t>Chain</t>
-        </is>
-      </c>
-      <c r="G139" t="n">
-        <v>300</v>
-      </c>
-      <c r="H139" t="n">
-        <v>251</v>
-      </c>
-      <c r="I139" t="n">
-        <v>0.8366666666666667</v>
-      </c>
-      <c r="J139" t="inlineStr"/>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>ProntoQA</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D140" t="n">
-        <v>8</v>
-      </c>
-      <c r="E140" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/ProntoQA__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F140" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="G140" t="n">
-        <v>0</v>
-      </c>
-      <c r="H140" t="n">
-        <v>0</v>
-      </c>
-      <c r="I140" t="n">
-        <v>0</v>
-      </c>
-      <c r="J140" t="inlineStr"/>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>ProntoQA</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D141" t="n">
-        <v>8</v>
-      </c>
-      <c r="E141" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/ProntoQA__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F141" t="inlineStr">
-        <is>
-          <t>Y-shaped</t>
-        </is>
-      </c>
-      <c r="G141" t="n">
-        <v>0</v>
-      </c>
-      <c r="H141" t="n">
-        <v>0</v>
-      </c>
-      <c r="I141" t="n">
-        <v>0</v>
-      </c>
-      <c r="J141" t="inlineStr"/>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>ProofWriter</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D142" t="n">
-        <v>8</v>
-      </c>
-      <c r="E142" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/ProofWriter__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F142" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="G142" t="n">
-        <v>300</v>
-      </c>
-      <c r="H142" t="n">
-        <v>247</v>
-      </c>
-      <c r="I142" t="n">
-        <v>0.8233333333333334</v>
-      </c>
-      <c r="J142" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>ProofWriter</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D143" t="n">
-        <v>8</v>
-      </c>
-      <c r="E143" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/ProofWriter__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F143" t="inlineStr">
-        <is>
-          <t>Block</t>
-        </is>
-      </c>
-      <c r="G143" t="n">
-        <v>0</v>
-      </c>
-      <c r="H143" t="n">
-        <v>0</v>
-      </c>
-      <c r="I143" t="n">
-        <v>0</v>
-      </c>
-      <c r="J143" t="inlineStr"/>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>ProofWriter</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D144" t="n">
-        <v>8</v>
-      </c>
-      <c r="E144" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/ProofWriter__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F144" t="inlineStr">
-        <is>
-          <t>Chain</t>
-        </is>
-      </c>
-      <c r="G144" t="n">
-        <v>300</v>
-      </c>
-      <c r="H144" t="n">
-        <v>247</v>
-      </c>
-      <c r="I144" t="n">
-        <v>0.8233333333333334</v>
-      </c>
-      <c r="J144" t="inlineStr"/>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>ProofWriter</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D145" t="n">
-        <v>8</v>
-      </c>
-      <c r="E145" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/ProofWriter__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F145" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="G145" t="n">
-        <v>0</v>
-      </c>
-      <c r="H145" t="n">
-        <v>0</v>
-      </c>
-      <c r="I145" t="n">
-        <v>0</v>
-      </c>
-      <c r="J145" t="inlineStr"/>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>ProofWriter</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D146" t="n">
-        <v>8</v>
-      </c>
-      <c r="E146" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/ProofWriter__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F146" t="inlineStr">
-        <is>
-          <t>Y-shaped</t>
-        </is>
-      </c>
-      <c r="G146" t="n">
-        <v>0</v>
-      </c>
-      <c r="H146" t="n">
-        <v>0</v>
-      </c>
-      <c r="I146" t="n">
-        <v>0</v>
-      </c>
-      <c r="J146" t="inlineStr"/>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>gsm8k</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D147" t="n">
-        <v>8</v>
-      </c>
-      <c r="E147" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/gsm8k__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F147" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="G147" t="n">
-        <v>300</v>
-      </c>
-      <c r="H147" t="n">
-        <v>256</v>
-      </c>
-      <c r="I147" t="n">
-        <v>0.8533333333333334</v>
-      </c>
-      <c r="J147" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>gsm8k</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D148" t="n">
-        <v>8</v>
-      </c>
-      <c r="E148" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/gsm8k__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F148" t="inlineStr">
-        <is>
-          <t>Block</t>
-        </is>
-      </c>
-      <c r="G148" t="n">
-        <v>0</v>
-      </c>
-      <c r="H148" t="n">
-        <v>0</v>
-      </c>
-      <c r="I148" t="n">
-        <v>0</v>
-      </c>
-      <c r="J148" t="inlineStr"/>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>gsm8k</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D149" t="n">
-        <v>8</v>
-      </c>
-      <c r="E149" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/gsm8k__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F149" t="inlineStr">
-        <is>
-          <t>Chain</t>
-        </is>
-      </c>
-      <c r="G149" t="n">
-        <v>300</v>
-      </c>
-      <c r="H149" t="n">
-        <v>256</v>
-      </c>
-      <c r="I149" t="n">
-        <v>0.8533333333333334</v>
-      </c>
-      <c r="J149" t="inlineStr"/>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>gsm8k</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D150" t="n">
-        <v>8</v>
-      </c>
-      <c r="E150" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/gsm8k__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F150" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="G150" t="n">
-        <v>0</v>
-      </c>
-      <c r="H150" t="n">
-        <v>0</v>
-      </c>
-      <c r="I150" t="n">
-        <v>0</v>
-      </c>
-      <c r="J150" t="inlineStr"/>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>gsm8k</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D151" t="n">
-        <v>8</v>
-      </c>
-      <c r="E151" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/gsm8k__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F151" t="inlineStr">
-        <is>
-          <t>Y-shaped</t>
-        </is>
-      </c>
-      <c r="G151" t="n">
-        <v>0</v>
-      </c>
-      <c r="H151" t="n">
-        <v>0</v>
-      </c>
-      <c r="I151" t="n">
-        <v>0</v>
-      </c>
-      <c r="J151" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6552,7 +4128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6665,16 +4241,16 @@
         <v>300</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.7433333333333333</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0.8333333333333334</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -6689,10 +4265,10 @@
         <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="P2" t="n">
-        <v>0</v>
+        <v>0.7433333333333333</v>
       </c>
     </row>
     <row r="3">
@@ -6723,16 +4299,16 @@
         <v>300</v>
       </c>
       <c r="G3" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.7366666666666667</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.8333333333333334</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -6747,10 +4323,10 @@
         <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="P3" t="n">
-        <v>0</v>
+        <v>0.7366666666666667</v>
       </c>
     </row>
     <row r="4">
@@ -6781,16 +4357,16 @@
         <v>300</v>
       </c>
       <c r="G4" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.8566666666666667</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.8333333333333334</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -6805,10 +4381,10 @@
         <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="P4" t="n">
-        <v>0</v>
+        <v>0.8566666666666667</v>
       </c>
     </row>
     <row r="5">
@@ -6839,16 +4415,16 @@
         <v>300</v>
       </c>
       <c r="G5" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.7366666666666667</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.8333333333333334</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -6863,10 +4439,10 @@
         <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>0.7366666666666667</v>
       </c>
     </row>
     <row r="6">
@@ -6897,16 +4473,16 @@
         <v>300</v>
       </c>
       <c r="G6" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.7366666666666667</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>0.8333333333333334</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
@@ -6921,10 +4497,10 @@
         <v>0</v>
       </c>
       <c r="O6" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="P6" t="n">
-        <v>0</v>
+        <v>0.7366666666666667</v>
       </c>
     </row>
     <row r="7">
@@ -6961,28 +4537,28 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>300</v>
+      </c>
+      <c r="P7" t="n">
         <v>0.79</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -7013,16 +4589,16 @@
         <v>300</v>
       </c>
       <c r="G8" t="n">
-        <v>0.8466666666666667</v>
+        <v>0.86</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>0.8466666666666667</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
@@ -7037,10 +4613,10 @@
         <v>0</v>
       </c>
       <c r="O8" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="P8" t="n">
-        <v>0</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="9">
@@ -7071,16 +4647,16 @@
         <v>300</v>
       </c>
       <c r="G9" t="n">
-        <v>0.8433333333333334</v>
+        <v>0.8733333333333333</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0.8433333333333334</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -7095,10 +4671,10 @@
         <v>0</v>
       </c>
       <c r="O9" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="P9" t="n">
-        <v>0</v>
+        <v>0.8733333333333333</v>
       </c>
     </row>
     <row r="10">
@@ -7129,16 +4705,16 @@
         <v>300</v>
       </c>
       <c r="G10" t="n">
-        <v>0.82</v>
+        <v>0.8633333333333333</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>0.82</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
@@ -7153,10 +4729,10 @@
         <v>0</v>
       </c>
       <c r="O10" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="P10" t="n">
-        <v>0</v>
+        <v>0.8633333333333333</v>
       </c>
     </row>
     <row r="11">
@@ -7187,16 +4763,16 @@
         <v>300</v>
       </c>
       <c r="G11" t="n">
-        <v>0.84</v>
+        <v>0.87</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>0.84</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
@@ -7211,10 +4787,10 @@
         <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="P11" t="n">
-        <v>0</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="12">
@@ -7245,16 +4821,16 @@
         <v>300</v>
       </c>
       <c r="G12" t="n">
-        <v>0.8066666666666666</v>
+        <v>0.7566666666666667</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>0.8066666666666666</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
@@ -7269,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="O12" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="P12" t="n">
-        <v>0</v>
+        <v>0.7566666666666667</v>
       </c>
     </row>
     <row r="13">
@@ -7303,16 +4879,16 @@
         <v>300</v>
       </c>
       <c r="G13" t="n">
-        <v>0.8666666666666667</v>
+        <v>0.88</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>0.8666666666666667</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -7327,10 +4903,10 @@
         <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="P13" t="n">
-        <v>0</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="14">
@@ -7367,28 +4943,28 @@
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="n">
+        <v>300</v>
+      </c>
+      <c r="P14" t="n">
         <v>0.84</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -7425,28 +5001,28 @@
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
+        <v>300</v>
+      </c>
+      <c r="P15" t="n">
         <v>0.8566666666666667</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -7477,16 +5053,16 @@
         <v>300</v>
       </c>
       <c r="G16" t="n">
-        <v>0.85</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>0.85</v>
+        <v>0</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -7501,10 +5077,10 @@
         <v>0</v>
       </c>
       <c r="O16" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="P16" t="n">
-        <v>0</v>
+        <v>0.8333333333333334</v>
       </c>
     </row>
     <row r="17">
@@ -7535,16 +5111,16 @@
         <v>300</v>
       </c>
       <c r="G17" t="n">
-        <v>0.7733333333333333</v>
+        <v>0.73</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>0.7733333333333333</v>
+        <v>0</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -7559,10 +5135,10 @@
         <v>0</v>
       </c>
       <c r="O17" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="P17" t="n">
-        <v>0</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="18">
@@ -7593,16 +5169,16 @@
         <v>300</v>
       </c>
       <c r="G18" t="n">
-        <v>0.8366666666666667</v>
+        <v>0.8566666666666667</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>0.8366666666666667</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
@@ -7617,16 +5193,16 @@
         <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="P18" t="n">
-        <v>0</v>
+        <v>0.8566666666666667</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ProntoQA</t>
+          <t>ProofWriter</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -7644,23 +5220,23 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>embed_results/LogicalDeduction/k4/ProntoQA__LogicalDeduction_dev_k4_icl.json</t>
+          <t>embed_results/LogicalDeduction/k4/ProofWriter__LogicalDeduction_dev_k4_icl.json</t>
         </is>
       </c>
       <c r="F19" t="n">
         <v>300</v>
       </c>
       <c r="G19" t="n">
-        <v>0.8533333333333334</v>
+        <v>0.8566666666666667</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>0.8533333333333334</v>
+        <v>0</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
@@ -7675,706 +5251,10 @@
         <v>0</v>
       </c>
       <c r="O19" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="P19" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>ProofWriter</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>4</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k4/ProofWriter__LogicalDeduction_dev_k4_icl.json</t>
-        </is>
-      </c>
-      <c r="F20" t="n">
-        <v>300</v>
-      </c>
-      <c r="G20" t="n">
-        <v>0.8466666666666667</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" t="n">
-        <v>300</v>
-      </c>
-      <c r="J20" t="n">
-        <v>0.8466666666666667</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>gsm8k</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>4</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k4/gsm8k__LogicalDeduction_dev_k4_icl.json</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>300</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" t="n">
-        <v>300</v>
-      </c>
-      <c r="J21" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>AR-LSAT</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>6</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/AR-LSAT__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F22" t="n">
-        <v>300</v>
-      </c>
-      <c r="G22" t="n">
-        <v>0.7733333333333333</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" t="n">
-        <v>300</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0.7733333333333333</v>
-      </c>
-      <c r="K22" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" t="n">
-        <v>0</v>
-      </c>
-      <c r="M22" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" t="n">
-        <v>0</v>
-      </c>
-      <c r="O22" t="n">
-        <v>0</v>
-      </c>
-      <c r="P22" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>FOLIO</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>6</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/FOLIO__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F23" t="n">
-        <v>300</v>
-      </c>
-      <c r="G23" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" t="n">
-        <v>300</v>
-      </c>
-      <c r="J23" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="K23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>ProntoQA</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>6</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/ProntoQA__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F24" t="n">
-        <v>300</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0.8466666666666667</v>
-      </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" t="n">
-        <v>300</v>
-      </c>
-      <c r="J24" t="n">
-        <v>0.8466666666666667</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>ProofWriter</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>6</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/ProofWriter__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F25" t="n">
-        <v>300</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0.8466666666666667</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" t="n">
-        <v>300</v>
-      </c>
-      <c r="J25" t="n">
-        <v>0.8466666666666667</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" t="n">
-        <v>0</v>
-      </c>
-      <c r="O25" t="n">
-        <v>0</v>
-      </c>
-      <c r="P25" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>gsm8k</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>6</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k6/gsm8k__LogicalDeduction_dev_k6_icl.json</t>
-        </is>
-      </c>
-      <c r="F26" t="n">
-        <v>300</v>
-      </c>
-      <c r="G26" t="n">
-        <v>0.8466666666666667</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" t="n">
-        <v>300</v>
-      </c>
-      <c r="J26" t="n">
-        <v>0.8466666666666667</v>
-      </c>
-      <c r="K26" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" t="n">
-        <v>0</v>
-      </c>
-      <c r="M26" t="n">
-        <v>0</v>
-      </c>
-      <c r="N26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P26" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>AR-LSAT</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>8</v>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/AR-LSAT__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F27" t="n">
-        <v>300</v>
-      </c>
-      <c r="G27" t="n">
-        <v>0.8066666666666666</v>
-      </c>
-      <c r="H27" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" t="n">
-        <v>300</v>
-      </c>
-      <c r="J27" t="n">
-        <v>0.8066666666666666</v>
-      </c>
-      <c r="K27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>FOLIO</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>8</v>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/FOLIO__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F28" t="n">
-        <v>300</v>
-      </c>
-      <c r="G28" t="n">
-        <v>0.8133333333333334</v>
-      </c>
-      <c r="H28" t="n">
-        <v>0</v>
-      </c>
-      <c r="I28" t="n">
-        <v>300</v>
-      </c>
-      <c r="J28" t="n">
-        <v>0.8133333333333334</v>
-      </c>
-      <c r="K28" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" t="n">
-        <v>0</v>
-      </c>
-      <c r="M28" t="n">
-        <v>0</v>
-      </c>
-      <c r="N28" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" t="n">
-        <v>0</v>
-      </c>
-      <c r="P28" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>ProntoQA</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>8</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/ProntoQA__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F29" t="n">
-        <v>300</v>
-      </c>
-      <c r="G29" t="n">
-        <v>0.8366666666666667</v>
-      </c>
-      <c r="H29" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" t="n">
-        <v>300</v>
-      </c>
-      <c r="J29" t="n">
-        <v>0.8366666666666667</v>
-      </c>
-      <c r="K29" t="n">
-        <v>0</v>
-      </c>
-      <c r="L29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P29" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>ProofWriter</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>8</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/ProofWriter__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F30" t="n">
-        <v>300</v>
-      </c>
-      <c r="G30" t="n">
-        <v>0.8233333333333334</v>
-      </c>
-      <c r="H30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" t="n">
-        <v>300</v>
-      </c>
-      <c r="J30" t="n">
-        <v>0.8233333333333334</v>
-      </c>
-      <c r="K30" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" t="n">
-        <v>0</v>
-      </c>
-      <c r="M30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P30" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>gsm8k</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>LogicalDeduction</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>dev</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>8</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>embed_results/LogicalDeduction/k8/gsm8k__LogicalDeduction_dev_k8_icl.json</t>
-        </is>
-      </c>
-      <c r="F31" t="n">
-        <v>300</v>
-      </c>
-      <c r="G31" t="n">
-        <v>0.8533333333333334</v>
-      </c>
-      <c r="H31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" t="n">
-        <v>300</v>
-      </c>
-      <c r="J31" t="n">
-        <v>0.8533333333333334</v>
-      </c>
-      <c r="K31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M31" t="n">
-        <v>0</v>
-      </c>
-      <c r="N31" t="n">
-        <v>0</v>
-      </c>
-      <c r="O31" t="n">
-        <v>0</v>
-      </c>
-      <c r="P31" t="n">
-        <v>0</v>
+        <v>0.8566666666666667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>